<commit_message>
fix: resolve admin dashboard crash and align stat fields
</commit_message>
<xml_diff>
--- a/User Ids.xlsx
+++ b/User Ids.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Rishabh\App Development\rcsfabrics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4840924-600E-47DF-BD0B-BD2D342DD723}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB1F8E1F-4736-4BD1-B2E9-F8F1B6987E7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,24 +25,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
     <t>Role</t>
-  </si>
-  <si>
-    <t>rish6.jain@gmail.com</t>
-  </si>
-  <si>
-    <t>Admin</t>
   </si>
   <si>
     <t>Email</t>
   </si>
   <si>
     <t>Name</t>
-  </si>
-  <si>
-    <t>Rishabh Jain</t>
   </si>
 </sst>
 </file>
@@ -385,30 +376,19 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>2</v>
-      </c>
+      <c r="B2" s="2"/>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" xr:uid="{AD85036F-BD96-46A0-9EBC-A1AD13BEFA7C}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>